<commit_message>
docs(huawei): Health Kit application material with AppGallery release proof
</commit_message>
<xml_diff>
--- a/huawei/Application+Material+(for+Individual+Developers).xlsx
+++ b/huawei/Application+Material+(for+Individual+Developers).xlsx
@@ -393,7 +393,7 @@
     <t>The step count read scope is used to obtain the user's daily step count from Huawei Health and display it in Step Challenge. The step count is used to calculate the user's progress in step challenges and rankings.</t>
   </si>
   <si>
-    <t>Yes. The app is available in the France mainland.</t>
+    <t>Yes. The app is released on HUAWEI AppGallery in France (version 1.9.1, app ID 118922449).</t>
   </si>
   <si>
     <t>Commercial use.</t>
@@ -1431,7 +1431,11 @@
       <c r="A5" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="25"/>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>Step Challenge is released on HUAWEI AppGallery (France), version 1.9.1, app ID 118922449: https://appgallery.huawei.com/app/C118922449. Huawei Health support is announced in the app as "coming soon" and will be enabled once this scope is granted.</t>
+        </is>
+      </c>
     </row>
     <row r="6" spans="1:2" ht="62.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="19" t="s">

</xml_diff>